<commit_message>
Edificio Ciudad Nueva: año de construcción 1990 y retiro del WEB ID (D-102)
- WEB ID retirado de portada, condiciones, aviso legal, Excel y respuestas del asesor
  (barrido de PPTX con notas, PDF y Excel: 0 coincidencias)
- D-102: el WEB ID es interno (identifica al captador) y nunca va en piezas para clientes
- Año de construcción 1990 (36 años) en portada, resumen, superficies, condiciones y riesgos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gncsby71g9SW8JZEc88cEa
</commit_message>
<xml_diff>
--- a/projects/edificio-ciudad-nueva/entregables/Edificio_Ciudad_Nueva_Alquileres_Rentabilidad.xlsx
+++ b/projects/edificio-ciudad-nueva/entregables/Edificio_Ciudad_Nueva_Alquileres_Rentabilidad.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="288">
   <si>
     <t xml:space="preserve">Rentabilidad sobre el precio — tipo de cambio del día</t>
   </si>
@@ -282,7 +282,19 @@
     <t xml:space="preserve">Ingreso bruto anual / m² construidos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Referencias, no tasación: el edificio es usado (antigüedad no informada) y el costo de reposición no descuenta depreciación. El comparable es un precio de oferta sin superficie publicada.</t>
+    <t xml:space="preserve">Año de construcción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informado por el founder.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antigüedad en 2026 (años)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año del análisis − año de construcción.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencias, no tasación: el edificio es de 1990 y el costo de reposición no descuenta depreciación ni estado de conservación. El comparable es un precio de oferta sin superficie publicada.</t>
   </si>
   <si>
     <t xml:space="preserve">Proyección de alquiler a 5 años — tres escenarios (USD, TC del día constante)</t>
@@ -702,7 +714,7 @@
     <t xml:space="preserve">Dato confirmado</t>
   </si>
   <si>
-    <t xml:space="preserve">Founder (WEB ID 143028006-118).</t>
+    <t xml:space="preserve">Founder.</t>
   </si>
   <si>
     <t xml:space="preserve">Tipo de cambio del día (Gs por USD)</t>
@@ -1123,6 +1135,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="173" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="173" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1136,10 +1152,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1920,7 +1932,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -2073,7 +2085,7 @@
         <v>80</v>
       </c>
       <c r="B15" s="16" t="n">
-        <f aca="false">Parametros!$B$33/Parametros!$B$34</f>
+        <f aca="false">Parametros!$B$34/Parametros!$B$35</f>
         <v>72222.2222222222</v>
       </c>
       <c r="C15" s="6" t="s">
@@ -2092,9 +2104,33 @@
         <v>83</v>
       </c>
     </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <f aca="false">Parametros!$B$33</f>
+        <v>1990</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>84</v>
+      <c r="A18" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <f aca="false">2026-Parametros!$B$33</f>
+        <v>36</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2122,7 +2158,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2132,29 +2168,29 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="n">
+      <c r="A5" s="20" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="16" t="n">
@@ -2183,7 +2219,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="n">
+      <c r="A6" s="20" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="16" t="n">
@@ -2212,7 +2248,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="20" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="16" t="n">
@@ -2241,7 +2277,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="n">
+      <c r="A8" s="20" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="16" t="n">
@@ -2270,7 +2306,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="20" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="16" t="n">
@@ -2300,86 +2336,86 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B10" s="20" t="n">
+        <v>97</v>
+      </c>
+      <c r="B10" s="21" t="n">
         <f aca="false">SUM(B5:B9)</f>
         <v>218743.10871549</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="21" t="n">
         <f aca="false">SUM(C5:C9)</f>
         <v>149169.69884939</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="21" t="n">
         <f aca="false">SUM(D5:D9)</f>
         <v>227662.994599579</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="21" t="n">
         <f aca="false">SUM(E5:E9)</f>
         <v>155472.727470364</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="21" t="n">
         <f aca="false">SUM(F5:F9)</f>
         <v>241711.377804004</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="21" t="n">
         <f aca="false">SUM(G5:G9)</f>
         <v>165399.688708046</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B11" s="21" t="n">
+        <v>98</v>
+      </c>
+      <c r="B11" s="22" t="n">
         <f aca="false">Parametros!$B$17</f>
         <v>0.03</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="22" t="n">
         <f aca="false">Parametros!$B$18</f>
         <v>0.05</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="22" t="n">
         <f aca="false">Parametros!$B$19</f>
         <v>0.08</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="G15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B16" s="22" t="n">
+        <v>107</v>
+      </c>
+      <c r="B16" s="23" t="n">
         <f aca="false">AVERAGEIFS(Alquileres_Unidad!$H$5:$H$19,Alquileres_Unidad!$E$5:$E$19,"1 dormitorio")</f>
         <v>1158333.33333333</v>
       </c>
@@ -2395,16 +2431,16 @@
         <f aca="false">C16/B16-1</f>
         <v>1.58992805755396</v>
       </c>
-      <c r="F16" s="23" t="n">
+      <c r="F16" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$E$5:$E$19,"1 dormitorio")</f>
         <v>6</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B17" s="22" t="n">
+        <v>108</v>
+      </c>
+      <c r="B17" s="23" t="n">
         <f aca="false">AVERAGEIFS(Alquileres_Unidad!$H$5:$H$19,Alquileres_Unidad!$E$5:$E$19,"2 dormitorios")</f>
         <v>1516666.66666667</v>
       </c>
@@ -2420,14 +2456,14 @@
         <f aca="false">C17/B17-1</f>
         <v>0.384615384615385</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$E$5:$E$19,"2 dormitorios")</f>
         <v>6</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C18" s="11" t="n">
         <f aca="false">Parametros!$B$27</f>
@@ -2436,7 +2472,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2500,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2477,35 +2513,35 @@
         <v>32</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="21" t="n">
+        <v>115</v>
+      </c>
+      <c r="B5" s="22" t="n">
         <f aca="false">Parametros!$B$20</f>
         <v>0.02</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="22" t="n">
         <f aca="false">Parametros!$B$21</f>
         <v>0.035</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="22" t="n">
         <f aca="false">Parametros!$B$22</f>
         <v>0.05</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B6" s="16" t="n">
         <f aca="false">Parametros!$B$5*(1+B5)^5</f>
@@ -2522,7 +2558,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">B6-Parametros!$B$5</f>
@@ -2539,7 +2575,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B8" s="16" t="n">
         <f aca="false">-B6*Parametros!$B$16</f>
@@ -2556,7 +2592,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B9" s="24" t="n">
         <f aca="false">Proyeccion!C10</f>
@@ -2573,24 +2609,24 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="20" t="n">
+        <v>120</v>
+      </c>
+      <c r="B10" s="21" t="n">
         <f aca="false">B7+B8+B9</f>
         <v>178926.35984107</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="21" t="n">
         <f aca="false">C7+C8+C9</f>
         <v>213228.871231502</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="21" t="n">
         <f aca="false">D7+D8+D9</f>
         <v>252826.383989297</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">B10/Parametros!$B$5</f>
@@ -2607,12 +2643,12 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B14" s="16" t="n">
         <f aca="false">-Parametros!$B$5</f>
@@ -2629,7 +2665,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B15" s="16" t="n">
         <f aca="false">Proyeccion!C5</f>
@@ -2646,7 +2682,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B16" s="16" t="n">
         <f aca="false">Proyeccion!C6</f>
@@ -2663,7 +2699,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B17" s="16" t="n">
         <f aca="false">Proyeccion!C7</f>
@@ -2680,7 +2716,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B18" s="16" t="n">
         <f aca="false">Proyeccion!C8</f>
@@ -2697,7 +2733,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B19" s="16" t="n">
         <f aca="false">Proyeccion!C9+B6+B8</f>
@@ -2714,7 +2750,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B20" s="25" t="n">
         <f aca="false">IRR(B14:B19)</f>
@@ -2731,7 +2767,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2768,7 +2804,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2778,37 +2814,37 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>15</v>
@@ -2819,19 +2855,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G5" s="27" t="n">
         <f aca="false">IF(F5="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -2844,12 +2880,12 @@
         <f aca="false">H5/Parametros!$B$6</f>
         <v>263.435194942044</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="23" t="n">
         <f aca="false">H5*G5</f>
         <v>75000</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L5" s="6"/>
     </row>
@@ -2858,19 +2894,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>138</v>
-      </c>
       <c r="D6" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G6" s="27" t="n">
         <f aca="false">IF(F6="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -2883,12 +2919,12 @@
         <f aca="false">H6/Parametros!$B$6</f>
         <v>263.435194942044</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="23" t="n">
         <f aca="false">H6*G6</f>
         <v>75000</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L6" s="6"/>
     </row>
@@ -2897,19 +2933,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D7" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">IF(F7="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -2922,12 +2958,12 @@
         <f aca="false">H7/Parametros!$B$6</f>
         <v>210.748155953635</v>
       </c>
-      <c r="J7" s="22" t="n">
+      <c r="J7" s="23" t="n">
         <f aca="false">H7*G7</f>
         <v>60000</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L7" s="6"/>
     </row>
@@ -2936,19 +2972,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D8" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="G8" s="27" t="n">
         <f aca="false">IF(F8="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -2961,12 +2997,12 @@
         <f aca="false">H8/Parametros!$B$6</f>
         <v>193.185809624166</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="23" t="n">
         <f aca="false">H8*G8</f>
         <v>55000</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L8" s="6"/>
     </row>
@@ -2975,19 +3011,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G9" s="27" t="n">
         <f aca="false">IF(F9="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3000,12 +3036,12 @@
         <f aca="false">H9/Parametros!$B$6</f>
         <v>280.997541271514</v>
       </c>
-      <c r="J9" s="22" t="n">
+      <c r="J9" s="23" t="n">
         <f aca="false">H9*G9</f>
         <v>80000</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L9" s="6"/>
     </row>
@@ -3014,19 +3050,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G10" s="27" t="n">
         <f aca="false">IF(F10="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3039,12 +3075,12 @@
         <f aca="false">H10/Parametros!$B$6</f>
         <v>263.435194942044</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="23" t="n">
         <f aca="false">H10*G10</f>
         <v>75000</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L10" s="6"/>
     </row>
@@ -3053,19 +3089,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G11" s="27" t="n">
         <f aca="false">IF(F11="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3078,12 +3114,12 @@
         <f aca="false">H11/Parametros!$B$6</f>
         <v>263.435194942044</v>
       </c>
-      <c r="J11" s="22" t="n">
+      <c r="J11" s="23" t="n">
         <f aca="false">H11*G11</f>
         <v>75000</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L11" s="6"/>
     </row>
@@ -3092,19 +3128,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G12" s="27" t="n">
         <f aca="false">IF(F12="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3117,12 +3153,12 @@
         <f aca="false">H12/Parametros!$B$6</f>
         <v>263.435194942044</v>
       </c>
-      <c r="J12" s="22" t="n">
+      <c r="J12" s="23" t="n">
         <f aca="false">H12*G12</f>
         <v>75000</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L12" s="6"/>
     </row>
@@ -3131,19 +3167,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>147</v>
-      </c>
       <c r="D13" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="G13" s="27" t="n">
         <f aca="false">IF(F13="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3156,12 +3192,12 @@
         <f aca="false">H13/Parametros!$B$6</f>
         <v>219.52932911837</v>
       </c>
-      <c r="J13" s="22" t="n">
+      <c r="J13" s="23" t="n">
         <f aca="false">H13*G13</f>
         <v>62500</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L13" s="6"/>
     </row>
@@ -3170,19 +3206,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D14" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="G14" s="27" t="n">
         <f aca="false">IF(F14="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3195,12 +3231,12 @@
         <f aca="false">H14/Parametros!$B$6</f>
         <v>228.310502283105</v>
       </c>
-      <c r="J14" s="22" t="n">
+      <c r="J14" s="23" t="n">
         <f aca="false">H14*G14</f>
         <v>65000</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L14" s="6"/>
     </row>
@@ -3209,19 +3245,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G15" s="27" t="n">
         <f aca="false">IF(F15="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3234,12 +3270,12 @@
         <f aca="false">H15/Parametros!$B$6</f>
         <v>280.997541271514</v>
       </c>
-      <c r="J15" s="22" t="n">
+      <c r="J15" s="23" t="n">
         <f aca="false">H15*G15</f>
         <v>80000</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L15" s="6"/>
     </row>
@@ -3248,19 +3284,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D16" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="G16" s="27" t="n">
         <f aca="false">IF(F16="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3273,12 +3309,12 @@
         <f aca="false">H16/Parametros!$B$6</f>
         <v>210.748155953635</v>
       </c>
-      <c r="J16" s="22" t="n">
+      <c r="J16" s="23" t="n">
         <f aca="false">H16*G16</f>
         <v>60000</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L16" s="6"/>
     </row>
@@ -3287,19 +3323,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D17" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="G17" s="27" t="n">
         <f aca="false">IF(F17="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3312,12 +3348,12 @@
         <f aca="false">H17/Parametros!$B$6</f>
         <v>158.061116965227</v>
       </c>
-      <c r="J17" s="22" t="n">
+      <c r="J17" s="23" t="n">
         <f aca="false">H17*G17</f>
         <v>45000</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L17" s="6"/>
     </row>
@@ -3326,19 +3362,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="G18" s="27" t="n">
         <f aca="false">IF(F18="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3351,15 +3387,15 @@
         <f aca="false">H18/Parametros!$B$6</f>
         <v>122.936424306287</v>
       </c>
-      <c r="J18" s="22" t="n">
+      <c r="J18" s="23" t="n">
         <f aca="false">H18*G18</f>
         <v>70000</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3367,19 +3403,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="G19" s="27" t="n">
         <f aca="false">IF(F19="Departamento",Parametros!$B$9,Parametros!$B$10)</f>
@@ -3392,20 +3428,20 @@
         <f aca="false">H19/Parametros!$B$6</f>
         <v>210.748155953635</v>
       </c>
-      <c r="J19" s="22" t="n">
+      <c r="J19" s="23" t="n">
         <f aca="false">H19*G19</f>
         <v>120000</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G20" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="H20" s="29" t="n">
         <f aca="false">SUM(H5:H19)</f>
@@ -3422,12 +3458,12 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -3457,7 +3493,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,16 +3506,16 @@
         <v>32</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>15</v>
@@ -3487,12 +3523,12 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$E$5:$E$19,"1 dormitorio")</f>
         <v>6</v>
       </c>
@@ -3507,12 +3543,12 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$E$5:$E$19,"2 dormitorios")</f>
         <v>6</v>
       </c>
@@ -3527,12 +3563,12 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$E$5:$E$19,"3 dormitorios")</f>
         <v>1</v>
       </c>
@@ -3547,12 +3583,12 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$F$5:$F$19,"Local comercial")</f>
         <v>0</v>
       </c>
@@ -3565,17 +3601,17 @@
         <v>Revisar</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B9" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$F$5:$F$19,"Cochera")</f>
         <v>1</v>
       </c>
@@ -3590,12 +3626,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$F$5:$F$19,"Cochera y departamento")</f>
         <v>1</v>
       </c>
@@ -3610,7 +3646,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">Alquileres_Unidad!$H$20</f>
@@ -3619,7 +3655,7 @@
       <c r="C12" s="28" t="n">
         <v>19550000</v>
       </c>
-      <c r="D12" s="22" t="n">
+      <c r="D12" s="23" t="n">
         <f aca="false">B12-C12</f>
         <v>0</v>
       </c>
@@ -3630,36 +3666,36 @@
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="F15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="B16" s="23" t="n">
+        <v>142</v>
+      </c>
+      <c r="B16" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$C$5:$C$19,A16)</f>
         <v>4</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="23" t="n">
         <f aca="false">SUMIFS(Alquileres_Unidad!$H$5:$H$19,Alquileres_Unidad!$C$5:$C$19,A16)</f>
         <v>5300000</v>
       </c>
@@ -3674,13 +3710,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B17" s="23" t="n">
+        <v>151</v>
+      </c>
+      <c r="B17" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$C$5:$C$19,A17)</f>
         <v>5</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="23" t="n">
         <f aca="false">SUMIFS(Alquileres_Unidad!$H$5:$H$19,Alquileres_Unidad!$C$5:$C$19,A17)</f>
         <v>7350000</v>
       </c>
@@ -3695,13 +3731,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B18" s="23" t="n">
+        <v>157</v>
+      </c>
+      <c r="B18" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$C$5:$C$19,A18)</f>
         <v>2</v>
       </c>
-      <c r="C18" s="22" t="n">
+      <c r="C18" s="23" t="n">
         <f aca="false">SUMIFS(Alquileres_Unidad!$H$5:$H$19,Alquileres_Unidad!$C$5:$C$19,A18)</f>
         <v>2900000</v>
       </c>
@@ -3716,13 +3752,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="B19" s="23" t="n">
+        <v>162</v>
+      </c>
+      <c r="B19" s="19" t="n">
         <f aca="false">COUNTIFS(Alquileres_Unidad!$C$5:$C$19,A19)</f>
         <v>4</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="23" t="n">
         <f aca="false">SUMIFS(Alquileres_Unidad!$H$5:$H$19,Alquileres_Unidad!$C$5:$C$19,A19)</f>
         <v>4000000</v>
       </c>
@@ -3737,9 +3773,9 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B20" s="19" t="n">
+        <v>190</v>
+      </c>
+      <c r="B20" s="20" t="n">
         <f aca="false">SUM(B16:B19)</f>
         <v>15</v>
       </c>
@@ -3782,50 +3818,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26"/>
       <c r="B6" s="26" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C6" s="26"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26"/>
       <c r="B7" s="26" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C7" s="26"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>1500000</v>
@@ -3833,10 +3869,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>1500000</v>
@@ -3844,10 +3880,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>1200000</v>
@@ -3855,10 +3891,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>1100000</v>
@@ -3867,16 +3903,16 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26"/>
       <c r="B12" s="26" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C12" s="26"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>1600000</v>
@@ -3884,10 +3920,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>1500000</v>
@@ -3895,10 +3931,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>1500000</v>
@@ -3906,10 +3942,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>1500000</v>
@@ -3917,10 +3953,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C17" s="28" t="n">
         <v>1250000</v>
@@ -3929,16 +3965,16 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26"/>
       <c r="B18" s="26" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C18" s="26"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C19" s="28" t="n">
         <v>1300000</v>
@@ -3946,10 +3982,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C20" s="28" t="n">
         <v>1600000</v>
@@ -3958,16 +3994,16 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26"/>
       <c r="B21" s="26" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C21" s="26"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C22" s="28" t="n">
         <v>1200000</v>
@@ -3975,10 +4011,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C23" s="28" t="n">
         <v>900000</v>
@@ -3986,10 +4022,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C24" s="28" t="n">
         <v>700000</v>
@@ -3997,10 +4033,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="26" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C25" s="28" t="n">
         <v>1200000</v>
@@ -4009,7 +4045,7 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="26"/>
       <c r="B26" s="26" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C26" s="28" t="n">
         <v>19550000</v>
@@ -4017,7 +4053,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="26" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B27" s="33" t="n">
         <v>6100</v>
@@ -4028,29 +4064,29 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4058,7 +4094,7 @@
         <v>340000</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C32" s="26" t="n">
         <v>3205</v>
@@ -4067,73 +4103,73 @@
         <v>19550000</v>
       </c>
       <c r="E32" s="26" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="26"/>
       <c r="B33" s="26" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C33" s="26" t="n">
         <v>2764</v>
       </c>
       <c r="D33" s="26"/>
       <c r="E33" s="26" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="26"/>
       <c r="B34" s="26" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C34" s="26" t="n">
         <v>1200</v>
       </c>
       <c r="D34" s="26"/>
       <c r="E34" s="26" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="26"/>
       <c r="B35" s="26" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C35" s="26"/>
       <c r="D35" s="26"/>
       <c r="E35" s="26" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="26"/>
       <c r="B36" s="26" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D36" s="26"/>
       <c r="E36" s="26"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="26" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C37" s="26"/>
       <c r="D37" s="26"/>
       <c r="E37" s="26" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -4152,7 +4188,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -4163,7 +4199,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4173,380 +4209,380 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B5" s="34" t="n">
         <v>340000</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B6" s="33" t="n">
         <v>5694</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B8" s="33" t="n">
         <v>6100</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B9" s="35" t="n">
         <v>0.05</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>0.1</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B11" s="35" t="n">
         <v>0.03</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>0.08</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B13" s="35" t="n">
         <v>0.05</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B14" s="34" t="n">
         <v>1200</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B15" s="35" t="n">
         <v>0.1</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="B16" s="37" t="n">
         <v>0.015</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B17" s="37" t="n">
         <v>0.03</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B18" s="37" t="n">
         <v>0.05</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B19" s="37" t="n">
         <v>0.08</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B20" s="37" t="n">
         <v>0.02</v>
       </c>
       <c r="C20" s="36" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B21" s="37" t="n">
         <v>0.035</v>
       </c>
       <c r="C21" s="36" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B22" s="37" t="n">
         <v>0.05</v>
       </c>
       <c r="C22" s="36" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B23" s="28" t="n">
         <v>3000000</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B24" s="28" t="n">
         <v>3200000</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B25" s="28" t="n">
         <v>2100000</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B26" s="28" t="n">
         <v>6300000</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B27" s="28" t="n">
         <v>2700000</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B28" s="38" t="n">
         <v>11</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B29" s="38" t="n">
         <v>31</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B30" s="33" t="n">
         <v>340</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4557,52 +4593,66 @@
         <v>1109</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="B32" s="34" t="n">
         <v>650</v>
       </c>
       <c r="C32" s="36" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="B33" s="34" t="n">
+        <v>84</v>
+      </c>
+      <c r="B33" s="18" t="n">
+        <v>1990</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B34" s="34" t="n">
         <v>650000</v>
       </c>
-      <c r="C33" s="10" t="s">
-        <v>265</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="B34" s="18" t="n">
+      <c r="C34" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B35" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="C34" s="10" t="s">
-        <v>265</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>268</v>
+      <c r="C35" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>